<commit_message>
docs(secs): workbook 追加項4 — CEID 17 no longer has an emit site
1f17067 removed the main-screen Tools button, which was the only emit site for
CEID 17 Enter Tool Page. The CEID sheet still marked it V. Flip row 18 to the
non-emitting shape (— / no Report / new remark), so the sheet now counts 55
unconditional + 1 conditional (78) + 236 never-sent = 292, matching firmware and
the interface spec. Update the two live status cells that carried the old totals
(檔首 2. CEID 表, and 功能!S1F23's "235 registered but never sent"), and add a
追加項4 block recording it. Historical per-version rows are left as written.

Edited by direct XML surgery, not openpyxl: the 功能 sheet carries two embedded
images that an openpyxl round-trip would silently drop. Only sheet1/2/4 differ;
the other 16 zip parts are byte-identical, including xl/drawings and xl/media.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SECS/SECS_GEM功能_Handler_20260804.xlsx
+++ b/docs/SECS/SECS_GEM功能_Handler_20260804.xlsx
@@ -951,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B148"/>
+  <dimension ref="A1:B154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" style="62" min="1" max="1"/>
@@ -1048,7 +1048,7 @@
       <c r="B10" s="26" t="inlineStr">
         <is>
           <t>整份改為 HT9045 字典的逐字複本(1-275 全數註冊，別名與 HT9045 逐字相同)。新增「本機發射」欄：52 個號碼本機真的會送(綠底並標 ★)，其餘 223 個已註冊但無發射點、永不送出。
-〔20260804 現況：CEID 字典已於 2026-08-03「追加項3」補齊為 1-292(第 1 版為 1-275)；發射點現為 56 個無條件發射(綠底、第 3 欄標 V)＋1 個條件發射(CEID 78，標「V(條件：出廠預設關閉)」)，合計 57 個，其餘 235 個已註冊但永不送出(第 3 欄標「—」)。本檔 CEID 工作表即為此數。⚠ 第 3 欄的欄名自 20260804 起為「HT-160」(原「本機發射」)，標記由「★」改為「V」—— 只是樣式，集合與底色完全未變。〕</t>
+〔20260804 現況：CEID 字典已於 2026-08-03「追加項3」補齊為 1-292(第 1 版為 1-275)；發射點現為 55 個無條件發射(綠底、第 3 欄標 V)＋1 個條件發射(CEID 78，標「V(條件：出廠預設關閉)」)，合計 56 個，其餘 236 個已註冊但永不送出(第 3 欄標「—」)。本檔 CEID 工作表即為此數。⚠ 第 3 欄的欄名自 20260804 起為「HT-160」(原「本機發射」)，標記由「★」改為「V」—— 只是樣式，集合與底色完全未變。⚠ 20260804 追加項4：CEID 17 Enter Tool Page 已由 V 改為「—」(主畫面 Tools 鍵移除、失去唯一發射點)，故無條件發射由 56 減為 55、合計由 57 減為 56、未發射由 235 增為 236，見第 35 項。〕</t>
         </is>
       </c>
     </row>
@@ -2609,6 +2609,68 @@
       <c r="B148" s="51" t="inlineStr">
         <is>
           <t>以 openpyxl 對第 6 版(commit 871bf08)逐格比對：差異共 59 格，全部落在 CEID!B1 / C1 / C 欄的 56 個發射標記，以及 ECID!C2 欄頭，無任何一格改到號碼、名稱、Report、備註或發射集合。CEID 表發射標記統計實測：V 56 個、V(條件：…) 1 個、— 235 個，合計 292。</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-04 第 6 版 追加項4(同日，承第 6 版)</t>
+        </is>
+      </c>
+      <c r="B150" s="40" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="34" t="inlineStr">
+        <is>
+          <t>依據韌體 Firmware</t>
+        </is>
+      </c>
+      <c r="B151" s="51" t="inlineStr">
+        <is>
+          <t>HT-160S 1.0.0.0, branch feat/iosetview-172-refactor (commit 1f17067)。本追加項為程式碼變更：移除主畫面工具列的 Tools 鍵，並修正 Message 鍵誤接警報視窗。建置：模擬版 -Clean exit 0；註銷 SOFT_SIMULATE 之真機版 -Full exit 0；還原後再 -Full exit 0；原始碼編碼檢查 166 檔通過。</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="34" t="inlineStr">
+        <is>
+          <t>⚠ 35. CEID 17 Enter Tool Page 自本版起不再發射(主畫面 Tools 鍵已移除)</t>
+        </is>
+      </c>
+      <c r="B152" s="51" t="inlineStr">
+        <is>
+          <t>本機主畫面工具列原有一顆 Tools 鍵，CEID 17 的唯一發射點就是它的按鈕處理常式。該鍵打開的是一片完全空白的視窗 —— HT-90XX 的 Tool 頁(使用者權限設定、警報碼產生)在本機分屬 UserRoleManager 與其他模組，從未移植過來，因此本日已將該按鈕整顆移除，其右側各鍵依序左移。
+• CEID 17 自本版起改列「已註冊但永不送出」：號碼與名稱仍保留在字典內(S1F23 / S1F24 全查仍會回它)，S2F35 連結仍會被接受(DRACK=0x00)，但永遠不會有 S6F11 送出。貴端若有訂閱請移除。
+• 無條件發射點由 56 減為 55，加上 CEID 78 的條件發射，合計由 57 減為 56；「已註冊但永不送出」由 235 增為 236。292 個號碼的總數不變。
+• 同時修正一個相關缺陷(不影響 SECS 介面)：Message 鍵原本開啟的是警報/回復視窗而非資料頁。在沒有警報時開啟該視窗會鳴警報蜂鳴器、把實體操作面板的按鍵交由該視窗處理，且面板 PAUSE 鍵會直接停下所有馬達。該鍵已改指向資料頁(目前為保留頁)。CEID 22 Enter Message Page 的發射時機不變 —— 仍是操作員按下 Message 鍵時送出，故 22 仍在發射清單內。</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="34" t="inlineStr">
+        <is>
+          <t>本次未變動 Unchanged</t>
+        </is>
+      </c>
+      <c r="B153" s="51" t="inlineStr">
+        <is>
+          <t>除 CEID 17 之外，其餘 291 個號碼的編號、名稱、語意與發射時機全部未變；SVID / ECID 的號碼、名稱、型別、可寫範圍未變；預設 Report 1(僅 1027 System Time)與 Report 2-7 未變；272-275 的 AMR 交握形狀未變；S5 警報目錄(481 筆)未變；Soter 輸出檔契約未變。本追加項只移除一顆從未有實際內容的操作介面按鈕。</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="34" t="inlineStr">
+        <is>
+          <t>追加項4 的驗證 Verification</t>
+        </is>
+      </c>
+      <c r="B154" s="51" t="inlineStr">
+        <is>
+          <t>1. 建置：模擬版 -Clean exit 0；註銷 SOFT_SIMULATE 之真機版 -Full exit 0；還原 SOFT_SIMULATE 後再 -Full exit 0；scripts/ops/check-ht160s-source-encoding.ps1 通過(166 檔)。
+2. 啟動實測：實際啟動重新建置的 EXE\ht160s.exe，各頁自我檢測回報 OPENED=Language,Product,Maintance,Teach,MotorTest,Offset,Speed,Message,Note，無例外；主畫面截圖確認工具列為 Language / Product / Maintance / Offset / Speed / Message / Monitor / Exit 共 8 鍵，Tools 已消失且無空位。
+3. 本表統計實測：CEID 工作表 V 55 個、V(條件：…) 1 個、— 236 個，合計 292。
+4. 規格書 HT160S_SECS_Interface_Spec_20260727.md / .html 已同步：§3.3.1 由 57 減為 56 並移除 CEID 17 一列，§3.3.2 由 235 增為 236 並新增 CEID 17 的逐條說明。</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2919,7 @@
   &lt;L [0] 
   &gt;
 .
-[20260730] 已實作(2026-07-30 新增)。S1F23 -&gt; S1F24 回 L,n{L,3{U4 CEID, A CENAME, L,m{U4 VID}}}。&lt;L[0]&gt; 全查回全部 292 個 CEID(與貴端現場機台的字典逐筆相同，含本機已註冊但不發射的 235 個)〔20260803:由 275 補齊為 292，見「第 4 版 追加項3」〕；指定 CEID 只回該幾筆；未註冊的 CEID 回 {CEID, '', L,0}(與 HT9045 同)。VID 清單由該 CEID 所連結的報表依序展開，順序與該事件 S6F11 內的排列一致，重複的 VID 不去除(一個 CEID 連兩張含相同 SVID 的報表時，S6F11 本來就會送兩次)。註：本訊息只是字典查詢，不等於訂閱 — 實際要收哪些事件仍由 S2F33 / S2F35 / S2F37 決定。</t>
+[20260730] 已實作(2026-07-30 新增)。S1F23 -&gt; S1F24 回 L,n{L,3{U4 CEID, A CENAME, L,m{U4 VID}}}。&lt;L[0]&gt; 全查回全部 292 個 CEID(與貴端現場機台的字典逐筆相同，含本機已註冊但不發射的 236 個)〔20260803:由 275 補齊為 292，見「第 4 版 追加項3」〕；指定 CEID 只回該幾筆；未註冊的 CEID 回 {CEID, '', L,0}(與 HT9045 同)。VID 清單由該 CEID 所連結的報表依序展開，順序與該事件 S6F11 內的排列一致，重複的 VID 不去除(一個 CEID 連兩張含相同 SVID 的報表時，S6F11 本來就會送兩次)。註：本訊息只是字典查詢，不等於訂閱 — 實際要收哪些事件仍由 S2F33 / S2F35 / S2F37 決定。</t>
         </is>
       </c>
     </row>
@@ -5173,27 +5235,23 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="67" t="n">
+      <c r="A18" s="69" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="68" t="inlineStr">
+      <c r="B18" s="70" t="inlineStr">
         <is>
           <t>Enter Tool Page</t>
         </is>
       </c>
-      <c r="C18" s="67" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D18" s="68" t="inlineStr">
-        <is>
-          <t>Report 1</t>
-        </is>
-      </c>
-      <c r="E18" s="68" t="inlineStr">
-        <is>
-          <t>進入 Tool 頁</t>
+      <c r="C18" s="69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D18" s="70" t="n"/>
+      <c r="E18" s="70" t="inlineStr">
+        <is>
+          <t>HT-160S 無 Tool 頁 —— 主畫面工具列的 Tools 鍵只會開出一片空白視窗，2026-08-04 已連同按鈕移除，本號碼自此不再發射(見「修訂說明」第 35 項)</t>
         </is>
       </c>
     </row>

</xml_diff>